<commit_message>
#316 Top Bits Command
- Added top bits command
- Fixed totalbits command configuration
- Added Lakea's capture Excel sheet
</commit_message>
<xml_diff>
--- a/Resources/Lakea Capture.xlsx
+++ b/Resources/Lakea Capture.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual Studio\Lakea-Stream-Assistant\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA90881-1701-48D5-B407-1ECDB8C9EE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6165776-5129-4DF2-BD3D-99668EBAA43A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lakeas Capture Modifiers" sheetId="2" r:id="rId1"/>
@@ -630,15 +630,15 @@
       </c>
       <c r="F5" s="3">
         <f>IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E5)&gt;SUM($C$20*E5),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E5),SUM($C$20*E5))</f>
-        <v>3.7209302325581417</v>
+        <v>15.348837209302326</v>
       </c>
       <c r="G5" s="3">
         <f>IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E5)&gt;SUM($C$20*E5),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E5),SUM($C$20*E5))</f>
-        <v>4.6511627906976774</v>
+        <v>19.186046511627907</v>
       </c>
       <c r="H5" s="3">
         <f>IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E5)&gt;SUM($C$20*E5),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E5),SUM($C$20*E5))</f>
-        <v>5.5813953488372121</v>
+        <v>23.02325581395349</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -668,7 +668,7 @@
       </c>
       <c r="R5" s="3">
         <f>IF(SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O5)&gt;SUM($C$20*J5),SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O5),SUM($C$20*J5))</f>
-        <v>3.8372093023255816</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -684,15 +684,15 @@
       </c>
       <c r="F6" s="3">
         <f t="shared" ref="F6:F69" si="0">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E6)&gt;SUM($C$20*E6),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E6),SUM($C$20*E6))</f>
-        <v>7.4418604651162834</v>
+        <v>30.697674418604652</v>
       </c>
       <c r="G6" s="3">
         <f t="shared" ref="G6:G69" si="1">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E6)&gt;SUM($C$20*E6),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E6),SUM($C$20*E6))</f>
-        <v>9.3023255813953547</v>
+        <v>38.372093023255815</v>
       </c>
       <c r="H6" s="3">
         <f t="shared" ref="H6:H69" si="2">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E6)&gt;SUM($C$20*E6),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E6),SUM($C$20*E6))</f>
-        <v>11.162790697674424</v>
+        <v>46.04651162790698</v>
       </c>
       <c r="J6">
         <f>J5 + 1</f>
@@ -724,7 +724,7 @@
       </c>
       <c r="R6" s="3">
         <f t="shared" ref="R6:R69" si="8">IF(SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O6)&gt;SUM($C$20*J6),SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O6),SUM($C$20*J6))</f>
-        <v>7.6744186046511631</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="7" spans="2:18" ht="30" x14ac:dyDescent="0.25">
@@ -740,15 +740,15 @@
       </c>
       <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>11.162790697674424</v>
+        <v>46.04651162790698</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" si="1"/>
-        <v>13.953488372093032</v>
+        <v>57.558139534883722</v>
       </c>
       <c r="H7" s="3">
         <f t="shared" si="2"/>
-        <v>16.744186046511636</v>
+        <v>69.069767441860478</v>
       </c>
       <c r="J7">
         <f t="shared" ref="J7:J70" si="10">J6 + 1</f>
@@ -780,7 +780,7 @@
       </c>
       <c r="R7" s="3">
         <f t="shared" si="8"/>
-        <v>11.511627906976745</v>
+        <v>10.050000000000001</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -790,15 +790,15 @@
       </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>14.883720930232567</v>
+        <v>61.395348837209305</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="1"/>
-        <v>18.604651162790709</v>
+        <v>76.744186046511629</v>
       </c>
       <c r="H8" s="3">
         <f t="shared" si="2"/>
-        <v>22.325581395348848</v>
+        <v>92.093023255813961</v>
       </c>
       <c r="J8">
         <f t="shared" si="10"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="R8" s="3">
         <f t="shared" si="8"/>
-        <v>15.348837209302326</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -846,15 +846,15 @@
       </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>18.604651162790709</v>
+        <v>76.744186046511629</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="1"/>
-        <v>23.255813953488385</v>
+        <v>95.930232558139537</v>
       </c>
       <c r="H9" s="3">
         <f t="shared" si="2"/>
-        <v>27.906976744186061</v>
+        <v>115.11627906976744</v>
       </c>
       <c r="J9">
         <f t="shared" si="10"/>
@@ -886,7 +886,7 @@
       </c>
       <c r="R9" s="3">
         <f t="shared" si="8"/>
-        <v>19.186046511627907</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -902,15 +902,15 @@
       </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>22.325581395348848</v>
+        <v>92.093023255813961</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="1"/>
-        <v>27.906976744186064</v>
+        <v>115.11627906976744</v>
       </c>
       <c r="H10" s="3">
         <f t="shared" si="2"/>
-        <v>33.488372093023273</v>
+        <v>138.13953488372096</v>
       </c>
       <c r="J10">
         <f t="shared" si="10"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="R10" s="3">
         <f t="shared" si="8"/>
-        <v>23.02325581395349</v>
+        <v>20.100000000000001</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -950,7 +950,7 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="E11">
         <f t="shared" si="9"/>
@@ -958,15 +958,15 @@
       </c>
       <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>26.046511627906991</v>
+        <v>107.44186046511628</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="1"/>
-        <v>32.558139534883743</v>
+        <v>134.30232558139534</v>
       </c>
       <c r="H11" s="3">
         <f t="shared" si="2"/>
-        <v>39.069767441860485</v>
+        <v>161.16279069767444</v>
       </c>
       <c r="J11">
         <f t="shared" si="10"/>
@@ -998,7 +998,7 @@
       </c>
       <c r="R11" s="3">
         <f t="shared" si="8"/>
-        <v>26.86046511627907</v>
+        <v>23.45</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -1014,15 +1014,15 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>29.767441860465134</v>
+        <v>122.79069767441861</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="1"/>
-        <v>37.209302325581419</v>
+        <v>153.48837209302326</v>
       </c>
       <c r="H12" s="3">
         <f t="shared" si="2"/>
-        <v>44.651162790697697</v>
+        <v>184.18604651162792</v>
       </c>
       <c r="J12">
         <f t="shared" si="10"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="R12" s="3">
         <f t="shared" si="8"/>
-        <v>30.697674418604652</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.25">
@@ -1070,15 +1070,15 @@
       </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>33.488372093023273</v>
+        <v>138.13953488372093</v>
       </c>
       <c r="G13" s="3">
         <f t="shared" si="1"/>
-        <v>41.860465116279094</v>
+        <v>172.67441860465118</v>
       </c>
       <c r="H13" s="3">
         <f t="shared" si="2"/>
-        <v>50.232558139534909</v>
+        <v>207.2093023255814</v>
       </c>
       <c r="J13">
         <f t="shared" si="10"/>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="R13" s="3">
         <f t="shared" si="8"/>
-        <v>34.534883720930232</v>
+        <v>30.150000000000002</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.25">
@@ -1126,15 +1126,15 @@
       </c>
       <c r="F14" s="3">
         <f t="shared" si="0"/>
-        <v>37.209302325581419</v>
+        <v>153.48837209302326</v>
       </c>
       <c r="G14" s="3">
         <f t="shared" si="1"/>
-        <v>46.51162790697677</v>
+        <v>191.86046511627907</v>
       </c>
       <c r="H14" s="3">
         <f t="shared" si="2"/>
-        <v>55.813953488372121</v>
+        <v>230.23255813953489</v>
       </c>
       <c r="J14">
         <f t="shared" si="10"/>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="R14" s="3">
         <f t="shared" si="8"/>
-        <v>38.372093023255815</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -1183,15 +1183,15 @@
       </c>
       <c r="F15" s="3">
         <f t="shared" si="0"/>
-        <v>40.930232558139558</v>
+        <v>168.83720930232559</v>
       </c>
       <c r="G15" s="3">
         <f t="shared" si="1"/>
-        <v>51.162790697674453</v>
+        <v>211.04651162790697</v>
       </c>
       <c r="H15" s="3">
         <f t="shared" si="2"/>
-        <v>61.395348837209333</v>
+        <v>253.2558139534884</v>
       </c>
       <c r="J15">
         <f t="shared" si="10"/>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="R15" s="3">
         <f t="shared" si="8"/>
-        <v>42.209302325581397</v>
+        <v>36.85</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -1233,15 +1233,15 @@
       </c>
       <c r="F16" s="3">
         <f t="shared" si="0"/>
-        <v>44.651162790697697</v>
+        <v>184.18604651162792</v>
       </c>
       <c r="G16" s="3">
         <f t="shared" si="1"/>
-        <v>55.813953488372128</v>
+        <v>230.23255813953489</v>
       </c>
       <c r="H16" s="3">
         <f t="shared" si="2"/>
-        <v>66.976744186046545</v>
+        <v>276.27906976744191</v>
       </c>
       <c r="J16">
         <f t="shared" si="10"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="R16" s="3">
         <f t="shared" si="8"/>
-        <v>46.04651162790698</v>
+        <v>40.200000000000003</v>
       </c>
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.25">
@@ -1289,15 +1289,15 @@
       </c>
       <c r="F17" s="3">
         <f t="shared" si="0"/>
-        <v>48.372093023255843</v>
+        <v>199.53488372093025</v>
       </c>
       <c r="G17" s="3">
         <f t="shared" si="1"/>
-        <v>60.465116279069804</v>
+        <v>249.41860465116281</v>
       </c>
       <c r="H17" s="3">
         <f t="shared" si="2"/>
-        <v>72.558139534883765</v>
+        <v>299.30232558139539</v>
       </c>
       <c r="J17">
         <f t="shared" si="10"/>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="R17" s="3">
         <f t="shared" si="8"/>
-        <v>49.883720930232563</v>
+        <v>43.550000000000004</v>
       </c>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
@@ -1345,15 +1345,15 @@
       </c>
       <c r="F18" s="3">
         <f t="shared" si="0"/>
-        <v>52.093023255813982</v>
+        <v>214.88372093023256</v>
       </c>
       <c r="G18" s="3">
         <f t="shared" si="1"/>
-        <v>65.116279069767486</v>
+        <v>268.60465116279067</v>
       </c>
       <c r="H18" s="3">
         <f t="shared" si="2"/>
-        <v>78.13953488372097</v>
+        <v>322.32558139534888</v>
       </c>
       <c r="J18">
         <f t="shared" si="10"/>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="R18" s="3">
         <f t="shared" si="8"/>
-        <v>53.720930232558139</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.25">
@@ -1393,7 +1393,7 @@
         <v>17</v>
       </c>
       <c r="C19">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E19">
         <f t="shared" si="9"/>
@@ -1401,15 +1401,15 @@
       </c>
       <c r="F19" s="3">
         <f t="shared" si="0"/>
-        <v>55.813953488372128</v>
+        <v>230.23255813953489</v>
       </c>
       <c r="G19" s="3">
         <f t="shared" si="1"/>
-        <v>69.767441860465155</v>
+        <v>287.7906976744186</v>
       </c>
       <c r="H19" s="3">
         <f t="shared" si="2"/>
-        <v>83.720930232558175</v>
+        <v>345.34883720930236</v>
       </c>
       <c r="J19">
         <f t="shared" si="10"/>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="R19" s="3">
         <f t="shared" si="8"/>
-        <v>57.558139534883722</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.25">
@@ -1457,15 +1457,15 @@
       </c>
       <c r="F20" s="3">
         <f t="shared" si="0"/>
-        <v>59.534883720930267</v>
+        <v>245.58139534883722</v>
       </c>
       <c r="G20" s="3">
         <f t="shared" si="1"/>
-        <v>74.418604651162838</v>
+        <v>306.97674418604652</v>
       </c>
       <c r="H20" s="3">
         <f t="shared" si="2"/>
-        <v>89.302325581395394</v>
+        <v>368.37209302325584</v>
       </c>
       <c r="J20">
         <f t="shared" si="10"/>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="R20" s="3">
         <f t="shared" si="8"/>
-        <v>61.395348837209305</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
@@ -1507,15 +1507,15 @@
       </c>
       <c r="F21" s="3">
         <f t="shared" si="0"/>
-        <v>63.255813953488406</v>
+        <v>260.93023255813955</v>
       </c>
       <c r="G21" s="3">
         <f t="shared" si="1"/>
-        <v>79.06976744186052</v>
+        <v>326.16279069767444</v>
       </c>
       <c r="H21" s="3">
         <f t="shared" si="2"/>
-        <v>94.883720930232613</v>
+        <v>391.39534883720933</v>
       </c>
       <c r="J21">
         <f t="shared" si="10"/>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="R21" s="3">
         <f t="shared" si="8"/>
-        <v>65.232558139534888</v>
+        <v>56.95</v>
       </c>
     </row>
     <row r="22" spans="2:18" x14ac:dyDescent="0.25">
@@ -1557,15 +1557,15 @@
       </c>
       <c r="F22" s="3">
         <f t="shared" si="0"/>
-        <v>66.976744186046545</v>
+        <v>276.27906976744185</v>
       </c>
       <c r="G22" s="3">
         <f t="shared" si="1"/>
-        <v>83.720930232558189</v>
+        <v>345.34883720930236</v>
       </c>
       <c r="H22" s="3">
         <f t="shared" si="2"/>
-        <v>100.46511627906982</v>
+        <v>414.41860465116281</v>
       </c>
       <c r="J22">
         <f t="shared" si="10"/>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="R22" s="3">
         <f t="shared" si="8"/>
-        <v>69.069767441860463</v>
+        <v>60.300000000000004</v>
       </c>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.25">
@@ -1607,15 +1607,15 @@
       </c>
       <c r="F23" s="3">
         <f t="shared" si="0"/>
-        <v>70.697674418604691</v>
+        <v>291.62790697674421</v>
       </c>
       <c r="G23" s="3">
         <f t="shared" si="1"/>
-        <v>88.372093023255871</v>
+        <v>364.53488372093022</v>
       </c>
       <c r="H23" s="3">
         <f t="shared" si="2"/>
-        <v>106.04651162790702</v>
+        <v>437.44186046511629</v>
       </c>
       <c r="J23">
         <f t="shared" si="10"/>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="R23" s="3">
         <f t="shared" si="8"/>
-        <v>72.906976744186053</v>
+        <v>63.65</v>
       </c>
     </row>
     <row r="24" spans="2:18" x14ac:dyDescent="0.25">
@@ -1657,15 +1657,15 @@
       </c>
       <c r="F24" s="3">
         <f t="shared" si="0"/>
-        <v>74.418604651162838</v>
+        <v>306.97674418604652</v>
       </c>
       <c r="G24" s="3">
         <f t="shared" si="1"/>
-        <v>93.02325581395354</v>
+        <v>383.72093023255815</v>
       </c>
       <c r="H24" s="3">
         <f t="shared" si="2"/>
-        <v>111.62790697674424</v>
+        <v>460.46511627906978</v>
       </c>
       <c r="J24">
         <f t="shared" si="10"/>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="R24" s="3">
         <f t="shared" si="8"/>
-        <v>76.744186046511629</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.25">
@@ -1707,15 +1707,15 @@
       </c>
       <c r="F25" s="3">
         <f t="shared" si="0"/>
-        <v>78.13953488372097</v>
+        <v>322.32558139534888</v>
       </c>
       <c r="G25" s="3">
         <f t="shared" si="1"/>
-        <v>97.674418604651223</v>
+        <v>402.90697674418607</v>
       </c>
       <c r="H25" s="3">
         <f t="shared" si="2"/>
-        <v>117.20930232558146</v>
+        <v>483.48837209302332</v>
       </c>
       <c r="J25">
         <f t="shared" si="10"/>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="R25" s="3">
         <f t="shared" si="8"/>
-        <v>80.581395348837219</v>
+        <v>70.350000000000009</v>
       </c>
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.25">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="F26" s="3">
         <f t="shared" si="0"/>
-        <v>81.860465116279116</v>
+        <v>337.67441860465118</v>
       </c>
       <c r="G26" s="3">
         <f t="shared" si="1"/>
-        <v>102.32558139534891</v>
+        <v>422.09302325581393</v>
       </c>
       <c r="H26" s="3">
         <f t="shared" si="2"/>
-        <v>122.79069767441867</v>
+        <v>506.5116279069768</v>
       </c>
       <c r="J26">
         <f t="shared" si="10"/>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="R26" s="3">
         <f t="shared" si="8"/>
-        <v>84.418604651162795</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.25">
@@ -1807,15 +1807,15 @@
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>85.581395348837262</v>
+        <v>353.02325581395348</v>
       </c>
       <c r="G27" s="3">
         <f t="shared" si="1"/>
-        <v>106.97674418604657</v>
+        <v>441.27906976744185</v>
       </c>
       <c r="H27" s="3">
         <f t="shared" si="2"/>
-        <v>128.37209302325587</v>
+        <v>529.53488372093022</v>
       </c>
       <c r="J27">
         <f t="shared" si="10"/>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="R27" s="3">
         <f t="shared" si="8"/>
-        <v>88.255813953488371</v>
+        <v>77.05</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
@@ -1857,15 +1857,15 @@
       </c>
       <c r="F28" s="3">
         <f t="shared" si="0"/>
-        <v>89.302325581395394</v>
+        <v>368.37209302325584</v>
       </c>
       <c r="G28" s="3">
         <f t="shared" si="1"/>
-        <v>111.62790697674426</v>
+        <v>460.46511627906978</v>
       </c>
       <c r="H28" s="3">
         <f t="shared" si="2"/>
-        <v>133.95348837209309</v>
+        <v>552.55813953488382</v>
       </c>
       <c r="J28">
         <f t="shared" si="10"/>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="R28" s="3">
         <f t="shared" si="8"/>
-        <v>92.093023255813961</v>
+        <v>80.400000000000006</v>
       </c>
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.25">
@@ -1907,15 +1907,15 @@
       </c>
       <c r="F29" s="3">
         <f t="shared" si="0"/>
-        <v>93.02325581395354</v>
+        <v>383.72093023255815</v>
       </c>
       <c r="G29" s="3">
         <f t="shared" si="1"/>
-        <v>116.27906976744194</v>
+        <v>479.6511627906977</v>
       </c>
       <c r="H29" s="3">
         <f t="shared" si="2"/>
-        <v>139.53488372093031</v>
+        <v>575.5813953488373</v>
       </c>
       <c r="J29">
         <f t="shared" si="10"/>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="R29" s="3">
         <f t="shared" si="8"/>
-        <v>95.930232558139537</v>
+        <v>83.75</v>
       </c>
     </row>
     <row r="30" spans="2:18" x14ac:dyDescent="0.25">
@@ -1957,15 +1957,15 @@
       </c>
       <c r="F30" s="3">
         <f t="shared" si="0"/>
-        <v>96.744186046511686</v>
+        <v>399.06976744186051</v>
       </c>
       <c r="G30" s="3">
         <f t="shared" si="1"/>
-        <v>120.93023255813961</v>
+        <v>498.83720930232562</v>
       </c>
       <c r="H30" s="3">
         <f t="shared" si="2"/>
-        <v>145.11627906976753</v>
+        <v>598.60465116279079</v>
       </c>
       <c r="J30">
         <f t="shared" si="10"/>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="R30" s="3">
         <f t="shared" si="8"/>
-        <v>99.767441860465127</v>
+        <v>87.100000000000009</v>
       </c>
     </row>
     <row r="31" spans="2:18" x14ac:dyDescent="0.25">
@@ -2007,15 +2007,15 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>100.46511627906983</v>
+        <v>414.41860465116281</v>
       </c>
       <c r="G31" s="3">
         <f t="shared" si="1"/>
-        <v>125.58139534883729</v>
+        <v>518.02325581395348</v>
       </c>
       <c r="H31" s="3">
         <f t="shared" si="2"/>
-        <v>150.69767441860472</v>
+        <v>621.62790697674427</v>
       </c>
       <c r="J31">
         <f t="shared" si="10"/>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="R31" s="3">
         <f t="shared" si="8"/>
-        <v>103.6046511627907</v>
+        <v>90.45</v>
       </c>
     </row>
     <row r="32" spans="2:18" x14ac:dyDescent="0.25">
@@ -2057,15 +2057,15 @@
       </c>
       <c r="F32" s="3">
         <f t="shared" si="0"/>
-        <v>104.18604651162796</v>
+        <v>429.76744186046511</v>
       </c>
       <c r="G32" s="3">
         <f t="shared" si="1"/>
-        <v>130.23255813953497</v>
+        <v>537.20930232558135</v>
       </c>
       <c r="H32" s="3">
         <f t="shared" si="2"/>
-        <v>156.27906976744194</v>
+        <v>644.65116279069775</v>
       </c>
       <c r="J32">
         <f t="shared" si="10"/>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="R32" s="3">
         <f t="shared" si="8"/>
-        <v>107.44186046511628</v>
+        <v>93.8</v>
       </c>
     </row>
     <row r="33" spans="5:18" x14ac:dyDescent="0.25">
@@ -2107,15 +2107,15 @@
       </c>
       <c r="F33" s="3">
         <f t="shared" si="0"/>
-        <v>107.90697674418611</v>
+        <v>445.11627906976747</v>
       </c>
       <c r="G33" s="3">
         <f t="shared" si="1"/>
-        <v>134.88372093023264</v>
+        <v>556.39534883720933</v>
       </c>
       <c r="H33" s="3">
         <f t="shared" si="2"/>
-        <v>161.86046511627916</v>
+        <v>667.67441860465124</v>
       </c>
       <c r="J33">
         <f t="shared" si="10"/>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="R33" s="3">
         <f t="shared" si="8"/>
-        <v>111.27906976744187</v>
+        <v>97.15</v>
       </c>
     </row>
     <row r="34" spans="5:18" x14ac:dyDescent="0.25">
@@ -2157,15 +2157,15 @@
       </c>
       <c r="F34" s="3">
         <f t="shared" si="0"/>
-        <v>111.62790697674426</v>
+        <v>460.46511627906978</v>
       </c>
       <c r="G34" s="3">
         <f t="shared" si="1"/>
-        <v>139.53488372093031</v>
+        <v>575.58139534883719</v>
       </c>
       <c r="H34" s="3">
         <f t="shared" si="2"/>
-        <v>167.44186046511635</v>
+        <v>690.69767441860472</v>
       </c>
       <c r="J34">
         <f t="shared" si="10"/>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="R34" s="3">
         <f t="shared" si="8"/>
-        <v>115.11627906976744</v>
+        <v>100.5</v>
       </c>
     </row>
     <row r="35" spans="5:18" x14ac:dyDescent="0.25">
@@ -2207,15 +2207,15 @@
       </c>
       <c r="F35" s="3">
         <f t="shared" si="0"/>
-        <v>115.34883720930239</v>
+        <v>475.81395348837214</v>
       </c>
       <c r="G35" s="3">
         <f t="shared" si="1"/>
-        <v>144.18604651162801</v>
+        <v>594.76744186046517</v>
       </c>
       <c r="H35" s="3">
         <f t="shared" si="2"/>
-        <v>173.02325581395357</v>
+        <v>713.7209302325582</v>
       </c>
       <c r="J35">
         <f t="shared" si="10"/>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="R35" s="3">
         <f t="shared" si="8"/>
-        <v>118.95348837209303</v>
+        <v>103.85000000000001</v>
       </c>
     </row>
     <row r="36" spans="5:18" x14ac:dyDescent="0.25">
@@ -2257,15 +2257,15 @@
       </c>
       <c r="F36" s="3">
         <f t="shared" si="0"/>
-        <v>119.06976744186053</v>
+        <v>491.16279069767444</v>
       </c>
       <c r="G36" s="3">
         <f t="shared" si="1"/>
-        <v>148.83720930232568</v>
+        <v>613.95348837209303</v>
       </c>
       <c r="H36" s="3">
         <f t="shared" si="2"/>
-        <v>178.60465116279079</v>
+        <v>736.74418604651169</v>
       </c>
       <c r="J36">
         <f t="shared" si="10"/>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="R36" s="3">
         <f t="shared" si="8"/>
-        <v>122.79069767441861</v>
+        <v>107.2</v>
       </c>
     </row>
     <row r="37" spans="5:18" x14ac:dyDescent="0.25">
@@ -2307,15 +2307,15 @@
       </c>
       <c r="F37" s="3">
         <f t="shared" si="0"/>
-        <v>122.79069767441868</v>
+        <v>506.51162790697674</v>
       </c>
       <c r="G37" s="3">
         <f t="shared" si="1"/>
-        <v>153.48837209302334</v>
+        <v>633.1395348837209</v>
       </c>
       <c r="H37" s="3">
         <f t="shared" si="2"/>
-        <v>184.18604651162801</v>
+        <v>759.76744186046517</v>
       </c>
       <c r="J37">
         <f t="shared" si="10"/>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="R37" s="3">
         <f t="shared" si="8"/>
-        <v>126.62790697674419</v>
+        <v>110.55</v>
       </c>
     </row>
     <row r="38" spans="5:18" x14ac:dyDescent="0.25">
@@ -2357,15 +2357,15 @@
       </c>
       <c r="F38" s="3">
         <f t="shared" si="0"/>
-        <v>126.51162790697681</v>
+        <v>521.8604651162791</v>
       </c>
       <c r="G38" s="3">
         <f t="shared" si="1"/>
-        <v>158.13953488372104</v>
+        <v>652.32558139534888</v>
       </c>
       <c r="H38" s="3">
         <f t="shared" si="2"/>
-        <v>189.76744186046523</v>
+        <v>782.79069767441865</v>
       </c>
       <c r="J38">
         <f t="shared" si="10"/>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="R38" s="3">
         <f t="shared" si="8"/>
-        <v>130.46511627906978</v>
+        <v>113.9</v>
       </c>
     </row>
     <row r="39" spans="5:18" x14ac:dyDescent="0.25">
@@ -2407,15 +2407,15 @@
       </c>
       <c r="F39" s="3">
         <f t="shared" si="0"/>
-        <v>130.23255813953497</v>
+        <v>537.20930232558146</v>
       </c>
       <c r="G39" s="3">
         <f t="shared" si="1"/>
-        <v>162.79069767441871</v>
+        <v>671.51162790697674</v>
       </c>
       <c r="H39" s="3">
         <f t="shared" si="2"/>
-        <v>195.34883720930242</v>
+        <v>805.81395348837214</v>
       </c>
       <c r="J39">
         <f t="shared" si="10"/>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="R39" s="3">
         <f t="shared" si="8"/>
-        <v>134.30232558139537</v>
+        <v>117.25</v>
       </c>
     </row>
     <row r="40" spans="5:18" x14ac:dyDescent="0.25">
@@ -2457,15 +2457,15 @@
       </c>
       <c r="F40" s="3">
         <f t="shared" si="0"/>
-        <v>133.95348837209309</v>
+        <v>552.55813953488371</v>
       </c>
       <c r="G40" s="3">
         <f t="shared" si="1"/>
-        <v>167.44186046511638</v>
+        <v>690.69767441860472</v>
       </c>
       <c r="H40" s="3">
         <f t="shared" si="2"/>
-        <v>200.93023255813964</v>
+        <v>828.83720930232562</v>
       </c>
       <c r="J40">
         <f t="shared" si="10"/>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="R40" s="3">
         <f t="shared" si="8"/>
-        <v>138.13953488372093</v>
+        <v>120.60000000000001</v>
       </c>
     </row>
     <row r="41" spans="5:18" x14ac:dyDescent="0.25">
@@ -2507,15 +2507,15 @@
       </c>
       <c r="F41" s="3">
         <f t="shared" si="0"/>
-        <v>137.67441860465124</v>
+        <v>567.90697674418607</v>
       </c>
       <c r="G41" s="3">
         <f t="shared" si="1"/>
-        <v>172.09302325581407</v>
+        <v>709.88372093023258</v>
       </c>
       <c r="H41" s="3">
         <f t="shared" si="2"/>
-        <v>206.51162790697686</v>
+        <v>851.8604651162791</v>
       </c>
       <c r="J41">
         <f t="shared" si="10"/>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="R41" s="3">
         <f t="shared" si="8"/>
-        <v>141.97674418604652</v>
+        <v>123.95</v>
       </c>
     </row>
     <row r="42" spans="5:18" x14ac:dyDescent="0.25">
@@ -2557,15 +2557,15 @@
       </c>
       <c r="F42" s="3">
         <f t="shared" si="0"/>
-        <v>141.39534883720938</v>
+        <v>583.25581395348843</v>
       </c>
       <c r="G42" s="3">
         <f t="shared" si="1"/>
-        <v>176.74418604651174</v>
+        <v>729.06976744186045</v>
       </c>
       <c r="H42" s="3">
         <f t="shared" si="2"/>
-        <v>212.09302325581405</v>
+        <v>874.88372093023258</v>
       </c>
       <c r="J42">
         <f t="shared" si="10"/>
@@ -2597,7 +2597,7 @@
       </c>
       <c r="R42" s="3">
         <f t="shared" si="8"/>
-        <v>145.81395348837211</v>
+        <v>127.3</v>
       </c>
     </row>
     <row r="43" spans="5:18" x14ac:dyDescent="0.25">
@@ -2607,15 +2607,15 @@
       </c>
       <c r="F43" s="3">
         <f t="shared" si="0"/>
-        <v>145.11627906976753</v>
+        <v>598.60465116279067</v>
       </c>
       <c r="G43" s="3">
         <f t="shared" si="1"/>
-        <v>181.39534883720941</v>
+        <v>748.25581395348843</v>
       </c>
       <c r="H43" s="3">
         <f t="shared" si="2"/>
-        <v>217.67441860465127</v>
+        <v>897.90697674418607</v>
       </c>
       <c r="J43">
         <f t="shared" si="10"/>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="R43" s="3">
         <f t="shared" si="8"/>
-        <v>149.65116279069767</v>
+        <v>130.65</v>
       </c>
     </row>
     <row r="44" spans="5:18" x14ac:dyDescent="0.25">
@@ -2657,15 +2657,15 @@
       </c>
       <c r="F44" s="3">
         <f t="shared" si="0"/>
-        <v>148.83720930232568</v>
+        <v>613.95348837209303</v>
       </c>
       <c r="G44" s="3">
         <f t="shared" si="1"/>
-        <v>186.04651162790708</v>
+        <v>767.44186046511629</v>
       </c>
       <c r="H44" s="3">
         <f t="shared" si="2"/>
-        <v>223.25581395348848</v>
+        <v>920.93023255813955</v>
       </c>
       <c r="J44">
         <f t="shared" si="10"/>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="R44" s="3">
         <f t="shared" si="8"/>
-        <v>153.48837209302326</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45" spans="5:18" x14ac:dyDescent="0.25">
@@ -2707,15 +2707,15 @@
       </c>
       <c r="F45" s="3">
         <f t="shared" si="0"/>
-        <v>152.55813953488382</v>
+        <v>629.30232558139539</v>
       </c>
       <c r="G45" s="3">
         <f t="shared" si="1"/>
-        <v>190.69767441860478</v>
+        <v>786.62790697674416</v>
       </c>
       <c r="H45" s="3">
         <f t="shared" si="2"/>
-        <v>228.8372093023257</v>
+        <v>943.95348837209315</v>
       </c>
       <c r="J45">
         <f t="shared" si="10"/>
@@ -2747,7 +2747,7 @@
       </c>
       <c r="R45" s="3">
         <f t="shared" si="8"/>
-        <v>157.32558139534885</v>
+        <v>137.35</v>
       </c>
     </row>
     <row r="46" spans="5:18" x14ac:dyDescent="0.25">
@@ -2757,15 +2757,15 @@
       </c>
       <c r="F46" s="3">
         <f t="shared" si="0"/>
-        <v>156.27906976744194</v>
+        <v>644.65116279069775</v>
       </c>
       <c r="G46" s="3">
         <f t="shared" si="1"/>
-        <v>195.34883720930245</v>
+        <v>805.81395348837214</v>
       </c>
       <c r="H46" s="3">
         <f t="shared" si="2"/>
-        <v>234.41860465116292</v>
+        <v>966.97674418604663</v>
       </c>
       <c r="J46">
         <f t="shared" si="10"/>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="R46" s="3">
         <f t="shared" si="8"/>
-        <v>161.16279069767444</v>
+        <v>140.70000000000002</v>
       </c>
     </row>
     <row r="47" spans="5:18" x14ac:dyDescent="0.25">
@@ -2807,15 +2807,15 @@
       </c>
       <c r="F47" s="3">
         <f t="shared" si="0"/>
-        <v>160.00000000000009</v>
+        <v>660</v>
       </c>
       <c r="G47" s="3">
         <f t="shared" si="1"/>
-        <v>200.00000000000011</v>
+        <v>825</v>
       </c>
       <c r="H47" s="3">
         <f t="shared" si="2"/>
-        <v>240.00000000000011</v>
+        <v>990.00000000000011</v>
       </c>
       <c r="J47">
         <f t="shared" si="10"/>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="R47" s="3">
         <f t="shared" si="8"/>
-        <v>165</v>
+        <v>144.05000000000001</v>
       </c>
     </row>
     <row r="48" spans="5:18" x14ac:dyDescent="0.25">
@@ -2857,15 +2857,15 @@
       </c>
       <c r="F48" s="3">
         <f t="shared" si="0"/>
-        <v>163.72093023255823</v>
+        <v>675.34883720930236</v>
       </c>
       <c r="G48" s="3">
         <f t="shared" si="1"/>
-        <v>204.65116279069781</v>
+        <v>844.18604651162786</v>
       </c>
       <c r="H48" s="3">
         <f t="shared" si="2"/>
-        <v>245.58139534883733</v>
+        <v>1013.0232558139536</v>
       </c>
       <c r="J48">
         <f t="shared" si="10"/>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="R48" s="3">
         <f t="shared" si="8"/>
-        <v>168.83720930232559</v>
+        <v>147.4</v>
       </c>
     </row>
     <row r="49" spans="5:18" x14ac:dyDescent="0.25">
@@ -2907,15 +2907,15 @@
       </c>
       <c r="F49" s="3">
         <f t="shared" si="0"/>
-        <v>167.44186046511638</v>
+        <v>690.69767441860472</v>
       </c>
       <c r="G49" s="3">
         <f t="shared" si="1"/>
-        <v>209.30232558139548</v>
+        <v>863.37209302325584</v>
       </c>
       <c r="H49" s="3">
         <f t="shared" si="2"/>
-        <v>251.16279069767455</v>
+        <v>1036.046511627907</v>
       </c>
       <c r="J49">
         <f t="shared" si="10"/>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="R49" s="3">
         <f t="shared" si="8"/>
-        <v>172.67441860465118</v>
+        <v>150.75</v>
       </c>
     </row>
     <row r="50" spans="5:18" x14ac:dyDescent="0.25">
@@ -2957,15 +2957,15 @@
       </c>
       <c r="F50" s="3">
         <f t="shared" si="0"/>
-        <v>171.16279069767452</v>
+        <v>706.04651162790697</v>
       </c>
       <c r="G50" s="3">
         <f t="shared" si="1"/>
-        <v>213.95348837209315</v>
+        <v>882.55813953488371</v>
       </c>
       <c r="H50" s="3">
         <f t="shared" si="2"/>
-        <v>256.74418604651174</v>
+        <v>1059.0697674418604</v>
       </c>
       <c r="J50">
         <f t="shared" si="10"/>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="R50" s="3">
         <f t="shared" si="8"/>
-        <v>176.51162790697674</v>
+        <v>154.1</v>
       </c>
     </row>
     <row r="51" spans="5:18" x14ac:dyDescent="0.25">
@@ -3007,15 +3007,15 @@
       </c>
       <c r="F51" s="3">
         <f t="shared" si="0"/>
-        <v>174.88372093023267</v>
+        <v>721.39534883720933</v>
       </c>
       <c r="G51" s="3">
         <f t="shared" si="1"/>
-        <v>218.60465116279084</v>
+        <v>901.74418604651169</v>
       </c>
       <c r="H51" s="3">
         <f t="shared" si="2"/>
-        <v>262.32558139534899</v>
+        <v>1082.0930232558139</v>
       </c>
       <c r="J51">
         <f t="shared" si="10"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="R51" s="3">
         <f t="shared" si="8"/>
-        <v>180.34883720930233</v>
+        <v>157.45000000000002</v>
       </c>
     </row>
     <row r="52" spans="5:18" x14ac:dyDescent="0.25">
@@ -3057,15 +3057,15 @@
       </c>
       <c r="F52" s="3">
         <f t="shared" si="0"/>
-        <v>178.60465116279079</v>
+        <v>736.74418604651169</v>
       </c>
       <c r="G52" s="3">
         <f t="shared" si="1"/>
-        <v>223.25581395348851</v>
+        <v>920.93023255813955</v>
       </c>
       <c r="H52" s="3">
         <f t="shared" si="2"/>
-        <v>267.90697674418618</v>
+        <v>1105.1162790697676</v>
       </c>
       <c r="J52">
         <f t="shared" si="10"/>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="R52" s="3">
         <f t="shared" si="8"/>
-        <v>184.18604651162792</v>
+        <v>160.80000000000001</v>
       </c>
     </row>
     <row r="53" spans="5:18" x14ac:dyDescent="0.25">
@@ -3107,15 +3107,15 @@
       </c>
       <c r="F53" s="3">
         <f t="shared" si="0"/>
-        <v>182.32558139534893</v>
+        <v>752.09302325581393</v>
       </c>
       <c r="G53" s="3">
         <f t="shared" si="1"/>
-        <v>227.90697674418618</v>
+        <v>940.11627906976742</v>
       </c>
       <c r="H53" s="3">
         <f t="shared" si="2"/>
-        <v>273.48837209302337</v>
+        <v>1128.1395348837211</v>
       </c>
       <c r="J53">
         <f t="shared" si="10"/>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="R53" s="3">
         <f t="shared" si="8"/>
-        <v>188.02325581395348</v>
+        <v>164.15</v>
       </c>
     </row>
     <row r="54" spans="5:18" x14ac:dyDescent="0.25">
@@ -3157,15 +3157,15 @@
       </c>
       <c r="F54" s="3">
         <f t="shared" si="0"/>
-        <v>186.04651162790708</v>
+        <v>767.44186046511629</v>
       </c>
       <c r="G54" s="3">
         <f t="shared" si="1"/>
-        <v>232.55813953488388</v>
+        <v>959.30232558139539</v>
       </c>
       <c r="H54" s="3">
         <f t="shared" si="2"/>
-        <v>279.06976744186062</v>
+        <v>1151.1627906976746</v>
       </c>
       <c r="J54">
         <f t="shared" si="10"/>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="R54" s="3">
         <f t="shared" si="8"/>
-        <v>191.86046511627907</v>
+        <v>167.5</v>
       </c>
     </row>
     <row r="55" spans="5:18" x14ac:dyDescent="0.25">
@@ -3207,15 +3207,15 @@
       </c>
       <c r="F55" s="3">
         <f t="shared" si="0"/>
-        <v>189.76744186046523</v>
+        <v>782.79069767441865</v>
       </c>
       <c r="G55" s="3">
         <f t="shared" si="1"/>
-        <v>237.20930232558155</v>
+        <v>978.48837209302326</v>
       </c>
       <c r="H55" s="3">
         <f t="shared" si="2"/>
-        <v>284.65116279069781</v>
+        <v>1174.1860465116281</v>
       </c>
       <c r="J55">
         <f t="shared" si="10"/>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="R55" s="3">
         <f t="shared" si="8"/>
-        <v>195.69767441860466</v>
+        <v>170.85</v>
       </c>
     </row>
     <row r="56" spans="5:18" x14ac:dyDescent="0.25">
@@ -3257,15 +3257,15 @@
       </c>
       <c r="F56" s="3">
         <f t="shared" si="0"/>
-        <v>193.48837209302337</v>
+        <v>798.13953488372101</v>
       </c>
       <c r="G56" s="3">
         <f t="shared" si="1"/>
-        <v>241.86046511627922</v>
+        <v>997.67441860465124</v>
       </c>
       <c r="H56" s="3">
         <f t="shared" si="2"/>
-        <v>290.23255813953506</v>
+        <v>1197.2093023255816</v>
       </c>
       <c r="J56">
         <f t="shared" si="10"/>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="R56" s="3">
         <f t="shared" si="8"/>
-        <v>199.53488372093025</v>
+        <v>174.20000000000002</v>
       </c>
     </row>
     <row r="57" spans="5:18" x14ac:dyDescent="0.25">
@@ -3307,15 +3307,15 @@
       </c>
       <c r="F57" s="3">
         <f t="shared" si="0"/>
-        <v>197.20930232558152</v>
+        <v>813.48837209302326</v>
       </c>
       <c r="G57" s="3">
         <f t="shared" si="1"/>
-        <v>246.51162790697691</v>
+        <v>1016.8604651162791</v>
       </c>
       <c r="H57" s="3">
         <f t="shared" si="2"/>
-        <v>295.81395348837225</v>
+        <v>1220.2325581395351</v>
       </c>
       <c r="J57">
         <f t="shared" si="10"/>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="R57" s="3">
         <f t="shared" si="8"/>
-        <v>203.37209302325581</v>
+        <v>177.55</v>
       </c>
     </row>
     <row r="58" spans="5:18" x14ac:dyDescent="0.25">
@@ -3357,15 +3357,15 @@
       </c>
       <c r="F58" s="3">
         <f t="shared" si="0"/>
-        <v>200.93023255813966</v>
+        <v>828.83720930232562</v>
       </c>
       <c r="G58" s="3">
         <f t="shared" si="1"/>
-        <v>251.16279069767458</v>
+        <v>1036.046511627907</v>
       </c>
       <c r="H58" s="3">
         <f t="shared" si="2"/>
-        <v>301.39534883720944</v>
+        <v>1243.2558139534885</v>
       </c>
       <c r="J58">
         <f t="shared" si="10"/>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="R58" s="3">
         <f t="shared" si="8"/>
-        <v>207.2093023255814</v>
+        <v>180.9</v>
       </c>
     </row>
     <row r="59" spans="5:18" x14ac:dyDescent="0.25">
@@ -3407,15 +3407,15 @@
       </c>
       <c r="F59" s="3">
         <f t="shared" si="0"/>
-        <v>204.65116279069778</v>
+        <v>844.18604651162798</v>
       </c>
       <c r="G59" s="3">
         <f t="shared" si="1"/>
-        <v>255.81395348837225</v>
+        <v>1055.2325581395348</v>
       </c>
       <c r="H59" s="3">
         <f t="shared" si="2"/>
-        <v>306.97674418604669</v>
+        <v>1266.279069767442</v>
       </c>
       <c r="J59">
         <f t="shared" si="10"/>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="R59" s="3">
         <f t="shared" si="8"/>
-        <v>211.04651162790699</v>
+        <v>184.25</v>
       </c>
     </row>
     <row r="60" spans="5:18" x14ac:dyDescent="0.25">
@@ -3457,15 +3457,15 @@
       </c>
       <c r="F60" s="3">
         <f t="shared" si="0"/>
-        <v>208.37209302325593</v>
+        <v>859.53488372093022</v>
       </c>
       <c r="G60" s="3">
         <f t="shared" si="1"/>
-        <v>260.46511627906995</v>
+        <v>1074.4186046511627</v>
       </c>
       <c r="H60" s="3">
         <f t="shared" si="2"/>
-        <v>312.55813953488388</v>
+        <v>1289.3023255813955</v>
       </c>
       <c r="J60">
         <f t="shared" si="10"/>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="R60" s="3">
         <f t="shared" si="8"/>
-        <v>214.88372093023256</v>
+        <v>187.6</v>
       </c>
     </row>
     <row r="61" spans="5:18" x14ac:dyDescent="0.25">
@@ -3507,15 +3507,15 @@
       </c>
       <c r="F61" s="3">
         <f t="shared" si="0"/>
-        <v>212.09302325581407</v>
+        <v>874.88372093023258</v>
       </c>
       <c r="G61" s="3">
         <f t="shared" si="1"/>
-        <v>265.11627906976759</v>
+        <v>1093.6046511627908</v>
       </c>
       <c r="H61" s="3">
         <f t="shared" si="2"/>
-        <v>318.13953488372107</v>
+        <v>1312.325581395349</v>
       </c>
       <c r="J61">
         <f t="shared" si="10"/>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="R61" s="3">
         <f t="shared" si="8"/>
-        <v>218.72093023255815</v>
+        <v>190.95000000000002</v>
       </c>
     </row>
     <row r="62" spans="5:18" x14ac:dyDescent="0.25">
@@ -3557,15 +3557,15 @@
       </c>
       <c r="F62" s="3">
         <f t="shared" si="0"/>
-        <v>215.81395348837222</v>
+        <v>890.23255813953494</v>
       </c>
       <c r="G62" s="3">
         <f t="shared" si="1"/>
-        <v>269.76744186046528</v>
+        <v>1112.7906976744187</v>
       </c>
       <c r="H62" s="3">
         <f t="shared" si="2"/>
-        <v>323.72093023255832</v>
+        <v>1335.3488372093025</v>
       </c>
       <c r="J62">
         <f t="shared" si="10"/>
@@ -3597,7 +3597,7 @@
       </c>
       <c r="R62" s="3">
         <f t="shared" si="8"/>
-        <v>222.55813953488374</v>
+        <v>194.3</v>
       </c>
     </row>
     <row r="63" spans="5:18" x14ac:dyDescent="0.25">
@@ -3607,15 +3607,15 @@
       </c>
       <c r="F63" s="3">
         <f t="shared" si="0"/>
-        <v>219.53488372093037</v>
+        <v>905.58139534883719</v>
       </c>
       <c r="G63" s="3">
         <f t="shared" si="1"/>
-        <v>274.41860465116298</v>
+        <v>1131.9767441860465</v>
       </c>
       <c r="H63" s="3">
         <f t="shared" si="2"/>
-        <v>329.30232558139551</v>
+        <v>1358.372093023256</v>
       </c>
       <c r="J63">
         <f t="shared" si="10"/>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="R63" s="3">
         <f t="shared" si="8"/>
-        <v>226.3953488372093</v>
+        <v>197.65</v>
       </c>
     </row>
     <row r="64" spans="5:18" x14ac:dyDescent="0.25">
@@ -3657,15 +3657,15 @@
       </c>
       <c r="F64" s="3">
         <f t="shared" si="0"/>
-        <v>223.25581395348851</v>
+        <v>920.93023255813955</v>
       </c>
       <c r="G64" s="3">
         <f t="shared" si="1"/>
-        <v>279.06976744186062</v>
+        <v>1151.1627906976744</v>
       </c>
       <c r="H64" s="3">
         <f t="shared" si="2"/>
-        <v>334.8837209302327</v>
+        <v>1381.3953488372094</v>
       </c>
       <c r="J64">
         <f t="shared" si="10"/>
@@ -3697,7 +3697,7 @@
       </c>
       <c r="R64" s="3">
         <f t="shared" si="8"/>
-        <v>230.23255813953489</v>
+        <v>201</v>
       </c>
     </row>
     <row r="65" spans="5:18" x14ac:dyDescent="0.25">
@@ -3707,15 +3707,15 @@
       </c>
       <c r="F65" s="3">
         <f t="shared" si="0"/>
-        <v>226.97674418604663</v>
+        <v>936.27906976744191</v>
       </c>
       <c r="G65" s="3">
         <f t="shared" si="1"/>
-        <v>283.72093023255832</v>
+        <v>1170.3488372093022</v>
       </c>
       <c r="H65" s="3">
         <f t="shared" si="2"/>
-        <v>340.46511627906995</v>
+        <v>1404.4186046511629</v>
       </c>
       <c r="J65">
         <f t="shared" si="10"/>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="R65" s="3">
         <f t="shared" si="8"/>
-        <v>234.06976744186048</v>
+        <v>204.35</v>
       </c>
     </row>
     <row r="66" spans="5:18" x14ac:dyDescent="0.25">
@@ -3757,15 +3757,15 @@
       </c>
       <c r="F66" s="3">
         <f t="shared" si="0"/>
-        <v>230.69767441860478</v>
+        <v>951.62790697674427</v>
       </c>
       <c r="G66" s="3">
         <f t="shared" si="1"/>
-        <v>288.37209302325601</v>
+        <v>1189.5348837209303</v>
       </c>
       <c r="H66" s="3">
         <f t="shared" si="2"/>
-        <v>346.04651162790714</v>
+        <v>1427.4418604651164</v>
       </c>
       <c r="J66">
         <f t="shared" si="10"/>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="R66" s="3">
         <f t="shared" si="8"/>
-        <v>237.90697674418607</v>
+        <v>207.70000000000002</v>
       </c>
     </row>
     <row r="67" spans="5:18" x14ac:dyDescent="0.25">
@@ -3807,15 +3807,15 @@
       </c>
       <c r="F67" s="3">
         <f t="shared" si="0"/>
-        <v>234.41860465116292</v>
+        <v>966.97674418604652</v>
       </c>
       <c r="G67" s="3">
         <f t="shared" si="1"/>
-        <v>293.02325581395365</v>
+        <v>1208.7209302325582</v>
       </c>
       <c r="H67" s="3">
         <f t="shared" si="2"/>
-        <v>351.62790697674438</v>
+        <v>1450.4651162790699</v>
       </c>
       <c r="J67">
         <f t="shared" si="10"/>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="R67" s="3">
         <f t="shared" si="8"/>
-        <v>241.74418604651163</v>
+        <v>211.05</v>
       </c>
     </row>
     <row r="68" spans="5:18" x14ac:dyDescent="0.25">
@@ -3857,15 +3857,15 @@
       </c>
       <c r="F68" s="3">
         <f t="shared" si="0"/>
-        <v>238.13953488372107</v>
+        <v>982.32558139534888</v>
       </c>
       <c r="G68" s="3">
         <f t="shared" si="1"/>
-        <v>297.67441860465135</v>
+        <v>1227.9069767441861</v>
       </c>
       <c r="H68" s="3">
         <f t="shared" si="2"/>
-        <v>357.20930232558158</v>
+        <v>1473.4883720930234</v>
       </c>
       <c r="J68">
         <f t="shared" si="10"/>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="R68" s="3">
         <f t="shared" si="8"/>
-        <v>245.58139534883722</v>
+        <v>214.4</v>
       </c>
     </row>
     <row r="69" spans="5:18" x14ac:dyDescent="0.25">
@@ -3907,15 +3907,15 @@
       </c>
       <c r="F69" s="3">
         <f t="shared" si="0"/>
-        <v>241.86046511627922</v>
+        <v>997.67441860465124</v>
       </c>
       <c r="G69" s="3">
         <f t="shared" si="1"/>
-        <v>302.32558139534905</v>
+        <v>1247.0930232558139</v>
       </c>
       <c r="H69" s="3">
         <f t="shared" si="2"/>
-        <v>362.79069767441877</v>
+        <v>1496.5116279069769</v>
       </c>
       <c r="J69">
         <f t="shared" si="10"/>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="R69" s="3">
         <f t="shared" si="8"/>
-        <v>249.41860465116281</v>
+        <v>217.75</v>
       </c>
     </row>
     <row r="70" spans="5:18" x14ac:dyDescent="0.25">
@@ -3957,15 +3957,15 @@
       </c>
       <c r="F70" s="3">
         <f t="shared" ref="F70:F124" si="12">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E70)&gt;SUM($C$20*E70),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$13)*E70),SUM($C$20*E70))</f>
-        <v>245.58139534883736</v>
+        <v>1013.0232558139535</v>
       </c>
       <c r="G70" s="3">
         <f t="shared" ref="G70:G124" si="13">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E70)&gt;SUM($C$20*E70),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$15)*E70),SUM($C$20*E70))</f>
-        <v>306.97674418604669</v>
+        <v>1266.2790697674418</v>
       </c>
       <c r="H70" s="3">
         <f t="shared" ref="H70:H124" si="14">IF(SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E70)&gt;SUM($C$20*E70),SUM((($C$12-(($C$11/3)/($C$10/3)))*$C$14)*E70),SUM($C$20*E70))</f>
-        <v>368.37209302325601</v>
+        <v>1519.5348837209303</v>
       </c>
       <c r="J70">
         <f t="shared" si="10"/>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="R70" s="3">
         <f t="shared" ref="R70:R124" si="20">IF(SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O70)&gt;SUM($C$20*J70),SUM((($C$12-(($C$19/3)/($C$10/3)))*$C$14)*O70),SUM($C$20*J70))</f>
-        <v>253.25581395348837</v>
+        <v>221.1</v>
       </c>
     </row>
     <row r="71" spans="5:18" x14ac:dyDescent="0.25">
@@ -4007,15 +4007,15 @@
       </c>
       <c r="F71" s="3">
         <f t="shared" si="12"/>
-        <v>249.30232558139551</v>
+        <v>1028.372093023256</v>
       </c>
       <c r="G71" s="3">
         <f t="shared" si="13"/>
-        <v>311.62790697674438</v>
+        <v>1285.4651162790699</v>
       </c>
       <c r="H71" s="3">
         <f t="shared" si="14"/>
-        <v>373.9534883720932</v>
+        <v>1542.5581395348838</v>
       </c>
       <c r="J71">
         <f t="shared" ref="J71:J124" si="22">J70 + 1</f>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="R71" s="3">
         <f t="shared" si="20"/>
-        <v>257.09302325581399</v>
+        <v>224.45000000000002</v>
       </c>
     </row>
     <row r="72" spans="5:18" x14ac:dyDescent="0.25">
@@ -4057,15 +4057,15 @@
       </c>
       <c r="F72" s="3">
         <f t="shared" si="12"/>
-        <v>253.02325581395363</v>
+        <v>1043.7209302325582</v>
       </c>
       <c r="G72" s="3">
         <f t="shared" si="13"/>
-        <v>316.27906976744208</v>
+        <v>1304.6511627906978</v>
       </c>
       <c r="H72" s="3">
         <f t="shared" si="14"/>
-        <v>379.53488372093045</v>
+        <v>1565.5813953488373</v>
       </c>
       <c r="J72">
         <f t="shared" si="22"/>
@@ -4097,7 +4097,7 @@
       </c>
       <c r="R72" s="3">
         <f t="shared" si="20"/>
-        <v>260.93023255813955</v>
+        <v>227.8</v>
       </c>
     </row>
     <row r="73" spans="5:18" x14ac:dyDescent="0.25">
@@ -4107,15 +4107,15 @@
       </c>
       <c r="F73" s="3">
         <f t="shared" si="12"/>
-        <v>256.7441860465118</v>
+        <v>1059.0697674418604</v>
       </c>
       <c r="G73" s="3">
         <f t="shared" si="13"/>
-        <v>320.93023255813972</v>
+        <v>1323.8372093023256</v>
       </c>
       <c r="H73" s="3">
         <f t="shared" si="14"/>
-        <v>385.11627906976764</v>
+        <v>1588.6046511627908</v>
       </c>
       <c r="J73">
         <f t="shared" si="22"/>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="R73" s="3">
         <f t="shared" si="20"/>
-        <v>264.76744186046511</v>
+        <v>231.15</v>
       </c>
     </row>
     <row r="74" spans="5:18" x14ac:dyDescent="0.25">
@@ -4157,15 +4157,15 @@
       </c>
       <c r="F74" s="3">
         <f t="shared" si="12"/>
-        <v>260.46511627906995</v>
+        <v>1074.4186046511629</v>
       </c>
       <c r="G74" s="3">
         <f t="shared" si="13"/>
-        <v>325.58139534883742</v>
+        <v>1343.0232558139535</v>
       </c>
       <c r="H74" s="3">
         <f t="shared" si="14"/>
-        <v>390.69767441860483</v>
+        <v>1611.6279069767443</v>
       </c>
       <c r="J74">
         <f t="shared" si="22"/>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="R74" s="3">
         <f t="shared" si="20"/>
-        <v>268.60465116279073</v>
+        <v>234.5</v>
       </c>
     </row>
     <row r="75" spans="5:18" x14ac:dyDescent="0.25">
@@ -4207,15 +4207,15 @@
       </c>
       <c r="F75" s="3">
         <f t="shared" si="12"/>
-        <v>264.18604651162804</v>
+        <v>1089.7674418604652</v>
       </c>
       <c r="G75" s="3">
         <f t="shared" si="13"/>
-        <v>330.23255813953512</v>
+        <v>1362.2093023255813</v>
       </c>
       <c r="H75" s="3">
         <f t="shared" si="14"/>
-        <v>396.27906976744208</v>
+        <v>1634.6511627906978</v>
       </c>
       <c r="J75">
         <f t="shared" si="22"/>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="R75" s="3">
         <f t="shared" si="20"/>
-        <v>272.44186046511629</v>
+        <v>237.85</v>
       </c>
     </row>
     <row r="76" spans="5:18" x14ac:dyDescent="0.25">
@@ -4257,15 +4257,15 @@
       </c>
       <c r="F76" s="3">
         <f t="shared" si="12"/>
-        <v>267.90697674418618</v>
+        <v>1105.1162790697674</v>
       </c>
       <c r="G76" s="3">
         <f t="shared" si="13"/>
-        <v>334.88372093023276</v>
+        <v>1381.3953488372094</v>
       </c>
       <c r="H76" s="3">
         <f t="shared" si="14"/>
-        <v>401.86046511627927</v>
+        <v>1657.6744186046512</v>
       </c>
       <c r="J76">
         <f t="shared" si="22"/>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="R76" s="3">
         <f t="shared" si="20"/>
-        <v>276.27906976744185</v>
+        <v>241.20000000000002</v>
       </c>
     </row>
     <row r="77" spans="5:18" x14ac:dyDescent="0.25">
@@ -4307,15 +4307,15 @@
       </c>
       <c r="F77" s="3">
         <f t="shared" si="12"/>
-        <v>271.62790697674433</v>
+        <v>1120.4651162790699</v>
       </c>
       <c r="G77" s="3">
         <f t="shared" si="13"/>
-        <v>339.53488372093045</v>
+        <v>1400.5813953488373</v>
       </c>
       <c r="H77" s="3">
         <f t="shared" si="14"/>
-        <v>407.44186046511646</v>
+        <v>1680.6976744186047</v>
       </c>
       <c r="J77">
         <f t="shared" si="22"/>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="R77" s="3">
         <f t="shared" si="20"/>
-        <v>280.11627906976747</v>
+        <v>244.55</v>
       </c>
     </row>
     <row r="78" spans="5:18" x14ac:dyDescent="0.25">
@@ -4357,15 +4357,15 @@
       </c>
       <c r="F78" s="3">
         <f t="shared" si="12"/>
-        <v>275.34883720930247</v>
+        <v>1135.8139534883721</v>
       </c>
       <c r="G78" s="3">
         <f t="shared" si="13"/>
-        <v>344.18604651162815</v>
+        <v>1419.7674418604652</v>
       </c>
       <c r="H78" s="3">
         <f t="shared" si="14"/>
-        <v>413.02325581395371</v>
+        <v>1703.7209302325582</v>
       </c>
       <c r="J78">
         <f t="shared" si="22"/>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="R78" s="3">
         <f t="shared" si="20"/>
-        <v>283.95348837209303</v>
+        <v>247.9</v>
       </c>
     </row>
     <row r="79" spans="5:18" x14ac:dyDescent="0.25">
@@ -4407,15 +4407,15 @@
       </c>
       <c r="F79" s="3">
         <f t="shared" si="12"/>
-        <v>279.06976744186062</v>
+        <v>1151.1627906976744</v>
       </c>
       <c r="G79" s="3">
         <f t="shared" si="13"/>
-        <v>348.83720930232579</v>
+        <v>1438.953488372093</v>
       </c>
       <c r="H79" s="3">
         <f t="shared" si="14"/>
-        <v>418.6046511627909</v>
+        <v>1726.7441860465117</v>
       </c>
       <c r="J79">
         <f t="shared" si="22"/>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="R79" s="3">
         <f t="shared" si="20"/>
-        <v>287.7906976744186</v>
+        <v>251.25</v>
       </c>
     </row>
     <row r="80" spans="5:18" x14ac:dyDescent="0.25">
@@ -4457,15 +4457,15 @@
       </c>
       <c r="F80" s="3">
         <f t="shared" si="12"/>
-        <v>282.79069767441877</v>
+        <v>1166.5116279069769</v>
       </c>
       <c r="G80" s="3">
         <f t="shared" si="13"/>
-        <v>353.48837209302349</v>
+        <v>1458.1395348837209</v>
       </c>
       <c r="H80" s="3">
         <f t="shared" si="14"/>
-        <v>424.18604651162809</v>
+        <v>1749.7674418604652</v>
       </c>
       <c r="J80">
         <f t="shared" si="22"/>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="R80" s="3">
         <f t="shared" si="20"/>
-        <v>291.62790697674421</v>
+        <v>254.6</v>
       </c>
     </row>
     <row r="81" spans="5:18" x14ac:dyDescent="0.25">
@@ -4507,15 +4507,15 @@
       </c>
       <c r="F81" s="3">
         <f t="shared" si="12"/>
-        <v>286.51162790697691</v>
+        <v>1181.8604651162791</v>
       </c>
       <c r="G81" s="3">
         <f t="shared" si="13"/>
-        <v>358.13953488372118</v>
+        <v>1477.3255813953488</v>
       </c>
       <c r="H81" s="3">
         <f t="shared" si="14"/>
-        <v>429.76744186046534</v>
+        <v>1772.7906976744187</v>
       </c>
       <c r="J81">
         <f t="shared" si="22"/>
@@ -4547,7 +4547,7 @@
       </c>
       <c r="R81" s="3">
         <f t="shared" si="20"/>
-        <v>295.46511627906978</v>
+        <v>257.95</v>
       </c>
     </row>
     <row r="82" spans="5:18" x14ac:dyDescent="0.25">
@@ -4557,15 +4557,15 @@
       </c>
       <c r="F82" s="3">
         <f t="shared" si="12"/>
-        <v>290.23255813953506</v>
+        <v>1197.2093023255813</v>
       </c>
       <c r="G82" s="3">
         <f t="shared" si="13"/>
-        <v>362.79069767441882</v>
+        <v>1496.5116279069769</v>
       </c>
       <c r="H82" s="3">
         <f t="shared" si="14"/>
-        <v>435.34883720930253</v>
+        <v>1795.8139534883721</v>
       </c>
       <c r="J82">
         <f t="shared" si="22"/>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="R82" s="3">
         <f t="shared" si="20"/>
-        <v>299.30232558139534</v>
+        <v>261.3</v>
       </c>
     </row>
     <row r="83" spans="5:18" x14ac:dyDescent="0.25">
@@ -4607,15 +4607,15 @@
       </c>
       <c r="F83" s="3">
         <f t="shared" si="12"/>
-        <v>293.9534883720932</v>
+        <v>1212.5581395348838</v>
       </c>
       <c r="G83" s="3">
         <f t="shared" si="13"/>
-        <v>367.44186046511652</v>
+        <v>1515.6976744186047</v>
       </c>
       <c r="H83" s="3">
         <f t="shared" si="14"/>
-        <v>440.93023255813978</v>
+        <v>1818.8372093023256</v>
       </c>
       <c r="J83">
         <f t="shared" si="22"/>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="R83" s="3">
         <f t="shared" si="20"/>
-        <v>303.13953488372096</v>
+        <v>264.65000000000003</v>
       </c>
     </row>
     <row r="84" spans="5:18" x14ac:dyDescent="0.25">
@@ -4657,15 +4657,15 @@
       </c>
       <c r="F84" s="3">
         <f t="shared" si="12"/>
-        <v>297.67441860465135</v>
+        <v>1227.9069767441861</v>
       </c>
       <c r="G84" s="3">
         <f t="shared" si="13"/>
-        <v>372.09302325581416</v>
+        <v>1534.8837209302326</v>
       </c>
       <c r="H84" s="3">
         <f t="shared" si="14"/>
-        <v>446.51162790697697</v>
+        <v>1841.8604651162791</v>
       </c>
       <c r="J84">
         <f t="shared" si="22"/>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="R84" s="3">
         <f t="shared" si="20"/>
-        <v>306.97674418604652</v>
+        <v>268</v>
       </c>
     </row>
     <row r="85" spans="5:18" x14ac:dyDescent="0.25">
@@ -4707,15 +4707,15 @@
       </c>
       <c r="F85" s="3">
         <f t="shared" si="12"/>
-        <v>301.3953488372095</v>
+        <v>1243.2558139534883</v>
       </c>
       <c r="G85" s="3">
         <f t="shared" si="13"/>
-        <v>376.74418604651186</v>
+        <v>1554.0697674418604</v>
       </c>
       <c r="H85" s="3">
         <f t="shared" si="14"/>
-        <v>452.09302325581416</v>
+        <v>1864.8837209302328</v>
       </c>
       <c r="J85">
         <f t="shared" si="22"/>
@@ -4747,7 +4747,7 @@
       </c>
       <c r="R85" s="3">
         <f t="shared" si="20"/>
-        <v>310.81395348837208</v>
+        <v>271.35000000000002</v>
       </c>
     </row>
     <row r="86" spans="5:18" x14ac:dyDescent="0.25">
@@ -4757,15 +4757,15 @@
       </c>
       <c r="F86" s="3">
         <f t="shared" si="12"/>
-        <v>305.11627906976764</v>
+        <v>1258.6046511627908</v>
       </c>
       <c r="G86" s="3">
         <f t="shared" si="13"/>
-        <v>381.39534883720955</v>
+        <v>1573.2558139534883</v>
       </c>
       <c r="H86" s="3">
         <f t="shared" si="14"/>
-        <v>457.67441860465141</v>
+        <v>1887.9069767441863</v>
       </c>
       <c r="J86">
         <f t="shared" si="22"/>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="R86" s="3">
         <f t="shared" si="20"/>
-        <v>314.6511627906977</v>
+        <v>274.7</v>
       </c>
     </row>
     <row r="87" spans="5:18" x14ac:dyDescent="0.25">
@@ -4807,15 +4807,15 @@
       </c>
       <c r="F87" s="3">
         <f t="shared" si="12"/>
-        <v>308.83720930232579</v>
+        <v>1273.953488372093</v>
       </c>
       <c r="G87" s="3">
         <f t="shared" si="13"/>
-        <v>386.04651162790719</v>
+        <v>1592.4418604651164</v>
       </c>
       <c r="H87" s="3">
         <f t="shared" si="14"/>
-        <v>463.2558139534886</v>
+        <v>1910.9302325581398</v>
       </c>
       <c r="J87">
         <f t="shared" si="22"/>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="R87" s="3">
         <f t="shared" si="20"/>
-        <v>318.48837209302326</v>
+        <v>278.05</v>
       </c>
     </row>
     <row r="88" spans="5:18" x14ac:dyDescent="0.25">
@@ -4857,15 +4857,15 @@
       </c>
       <c r="F88" s="3">
         <f t="shared" si="12"/>
-        <v>312.55813953488388</v>
+        <v>1289.3023255813955</v>
       </c>
       <c r="G88" s="3">
         <f t="shared" si="13"/>
-        <v>390.69767441860489</v>
+        <v>1611.6279069767443</v>
       </c>
       <c r="H88" s="3">
         <f t="shared" si="14"/>
-        <v>468.83720930232585</v>
+        <v>1933.9534883720933</v>
       </c>
       <c r="J88">
         <f t="shared" si="22"/>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="R88" s="3">
         <f t="shared" si="20"/>
-        <v>322.32558139534888</v>
+        <v>281.40000000000003</v>
       </c>
     </row>
     <row r="89" spans="5:18" x14ac:dyDescent="0.25">
@@ -4907,15 +4907,15 @@
       </c>
       <c r="F89" s="3">
         <f t="shared" si="12"/>
-        <v>316.27906976744202</v>
+        <v>1304.6511627906978</v>
       </c>
       <c r="G89" s="3">
         <f t="shared" si="13"/>
-        <v>395.34883720930259</v>
+        <v>1630.8139534883721</v>
       </c>
       <c r="H89" s="3">
         <f t="shared" si="14"/>
-        <v>474.41860465116304</v>
+        <v>1956.9767441860467</v>
       </c>
       <c r="J89">
         <f t="shared" si="22"/>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="R89" s="3">
         <f t="shared" si="20"/>
-        <v>326.16279069767444</v>
+        <v>284.75</v>
       </c>
     </row>
     <row r="90" spans="5:18" x14ac:dyDescent="0.25">
@@ -4957,15 +4957,15 @@
       </c>
       <c r="F90" s="3">
         <f t="shared" si="12"/>
-        <v>320.00000000000017</v>
+        <v>1320</v>
       </c>
       <c r="G90" s="3">
         <f t="shared" si="13"/>
-        <v>400.00000000000023</v>
+        <v>1650</v>
       </c>
       <c r="H90" s="3">
         <f t="shared" si="14"/>
-        <v>480.00000000000023</v>
+        <v>1980.0000000000002</v>
       </c>
       <c r="J90">
         <f t="shared" si="22"/>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="R90" s="3">
         <f t="shared" si="20"/>
-        <v>330</v>
+        <v>288.10000000000002</v>
       </c>
     </row>
     <row r="91" spans="5:18" x14ac:dyDescent="0.25">
@@ -5007,15 +5007,15 @@
       </c>
       <c r="F91" s="3">
         <f t="shared" si="12"/>
-        <v>323.72093023255832</v>
+        <v>1335.3488372093025</v>
       </c>
       <c r="G91" s="3">
         <f t="shared" si="13"/>
-        <v>404.65116279069792</v>
+        <v>1669.1860465116279</v>
       </c>
       <c r="H91" s="3">
         <f t="shared" si="14"/>
-        <v>485.58139534883748</v>
+        <v>2003.0232558139537</v>
       </c>
       <c r="J91">
         <f t="shared" si="22"/>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="R91" s="3">
         <f t="shared" si="20"/>
-        <v>333.83720930232562</v>
+        <v>291.45</v>
       </c>
     </row>
     <row r="92" spans="5:18" x14ac:dyDescent="0.25">
@@ -5057,15 +5057,15 @@
       </c>
       <c r="F92" s="3">
         <f t="shared" si="12"/>
-        <v>327.44186046511646</v>
+        <v>1350.6976744186047</v>
       </c>
       <c r="G92" s="3">
         <f t="shared" si="13"/>
-        <v>409.30232558139562</v>
+        <v>1688.3720930232557</v>
       </c>
       <c r="H92" s="3">
         <f t="shared" si="14"/>
-        <v>491.16279069767467</v>
+        <v>2026.0465116279072</v>
       </c>
       <c r="J92">
         <f t="shared" si="22"/>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="R92" s="3">
         <f t="shared" si="20"/>
-        <v>337.67441860465118</v>
+        <v>294.8</v>
       </c>
     </row>
     <row r="93" spans="5:18" x14ac:dyDescent="0.25">
@@ -5107,15 +5107,15 @@
       </c>
       <c r="F93" s="3">
         <f t="shared" si="12"/>
-        <v>331.16279069767461</v>
+        <v>1366.046511627907</v>
       </c>
       <c r="G93" s="3">
         <f t="shared" si="13"/>
-        <v>413.95348837209326</v>
+        <v>1707.5581395348838</v>
       </c>
       <c r="H93" s="3">
         <f t="shared" si="14"/>
-        <v>496.74418604651186</v>
+        <v>2049.0697674418607</v>
       </c>
       <c r="J93">
         <f t="shared" si="22"/>
@@ -5147,7 +5147,7 @@
       </c>
       <c r="R93" s="3">
         <f t="shared" si="20"/>
-        <v>341.51162790697674</v>
+        <v>298.15000000000003</v>
       </c>
     </row>
     <row r="94" spans="5:18" x14ac:dyDescent="0.25">
@@ -5157,15 +5157,15 @@
       </c>
       <c r="F94" s="3">
         <f t="shared" si="12"/>
-        <v>334.88372093023276</v>
+        <v>1381.3953488372094</v>
       </c>
       <c r="G94" s="3">
         <f t="shared" si="13"/>
-        <v>418.60465116279096</v>
+        <v>1726.7441860465117</v>
       </c>
       <c r="H94" s="3">
         <f t="shared" si="14"/>
-        <v>502.3255813953491</v>
+        <v>2072.0930232558139</v>
       </c>
       <c r="J94">
         <f t="shared" si="22"/>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="R94" s="3">
         <f t="shared" si="20"/>
-        <v>345.34883720930236</v>
+        <v>301.5</v>
       </c>
     </row>
     <row r="95" spans="5:18" x14ac:dyDescent="0.25">
@@ -5207,15 +5207,15 @@
       </c>
       <c r="F95" s="3">
         <f t="shared" si="12"/>
-        <v>338.6046511627909</v>
+        <v>1396.7441860465117</v>
       </c>
       <c r="G95" s="3">
         <f t="shared" si="13"/>
-        <v>423.25581395348865</v>
+        <v>1745.9302325581396</v>
       </c>
       <c r="H95" s="3">
         <f t="shared" si="14"/>
-        <v>507.9069767441863</v>
+        <v>2095.1162790697676</v>
       </c>
       <c r="J95">
         <f t="shared" si="22"/>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="R95" s="3">
         <f t="shared" si="20"/>
-        <v>349.18604651162792</v>
+        <v>304.85000000000002</v>
       </c>
     </row>
     <row r="96" spans="5:18" x14ac:dyDescent="0.25">
@@ -5257,15 +5257,15 @@
       </c>
       <c r="F96" s="3">
         <f t="shared" si="12"/>
-        <v>342.32558139534905</v>
+        <v>1412.0930232558139</v>
       </c>
       <c r="G96" s="3">
         <f t="shared" si="13"/>
-        <v>427.9069767441863</v>
+        <v>1765.1162790697674</v>
       </c>
       <c r="H96" s="3">
         <f t="shared" si="14"/>
-        <v>513.48837209302349</v>
+        <v>2118.1395348837209</v>
       </c>
       <c r="J96">
         <f t="shared" si="22"/>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="R96" s="3">
         <f t="shared" si="20"/>
-        <v>353.02325581395348</v>
+        <v>308.2</v>
       </c>
     </row>
     <row r="97" spans="5:18" x14ac:dyDescent="0.25">
@@ -5307,15 +5307,15 @@
       </c>
       <c r="F97" s="3">
         <f t="shared" si="12"/>
-        <v>346.04651162790719</v>
+        <v>1427.4418604651164</v>
       </c>
       <c r="G97" s="3">
         <f t="shared" si="13"/>
-        <v>432.55813953488399</v>
+        <v>1784.3023255813953</v>
       </c>
       <c r="H97" s="3">
         <f t="shared" si="14"/>
-        <v>519.06976744186068</v>
+        <v>2141.1627906976746</v>
       </c>
       <c r="J97">
         <f t="shared" si="22"/>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="R97" s="3">
         <f t="shared" si="20"/>
-        <v>356.8604651162791</v>
+        <v>311.55</v>
       </c>
     </row>
     <row r="98" spans="5:18" x14ac:dyDescent="0.25">
@@ -5357,15 +5357,15 @@
       </c>
       <c r="F98" s="3">
         <f t="shared" si="12"/>
-        <v>349.76744186046534</v>
+        <v>1442.7906976744187</v>
       </c>
       <c r="G98" s="3">
         <f t="shared" si="13"/>
-        <v>437.20930232558169</v>
+        <v>1803.4883720930234</v>
       </c>
       <c r="H98" s="3">
         <f t="shared" si="14"/>
-        <v>524.65116279069798</v>
+        <v>2164.1860465116279</v>
       </c>
       <c r="J98">
         <f t="shared" si="22"/>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="R98" s="3">
         <f t="shared" si="20"/>
-        <v>360.69767441860466</v>
+        <v>314.90000000000003</v>
       </c>
     </row>
     <row r="99" spans="5:18" x14ac:dyDescent="0.25">
@@ -5407,15 +5407,15 @@
       </c>
       <c r="F99" s="3">
         <f t="shared" si="12"/>
-        <v>353.48837209302349</v>
+        <v>1458.1395348837209</v>
       </c>
       <c r="G99" s="3">
         <f t="shared" si="13"/>
-        <v>441.86046511627933</v>
+        <v>1822.6744186046512</v>
       </c>
       <c r="H99" s="3">
         <f t="shared" si="14"/>
-        <v>530.23255813953517</v>
+        <v>2187.2093023255816</v>
       </c>
       <c r="J99">
         <f t="shared" si="22"/>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="R99" s="3">
         <f t="shared" si="20"/>
-        <v>364.53488372093022</v>
+        <v>318.25</v>
       </c>
     </row>
     <row r="100" spans="5:18" x14ac:dyDescent="0.25">
@@ -5457,15 +5457,15 @@
       </c>
       <c r="F100" s="3">
         <f t="shared" si="12"/>
-        <v>357.20930232558158</v>
+        <v>1473.4883720930234</v>
       </c>
       <c r="G100" s="3">
         <f t="shared" si="13"/>
-        <v>446.51162790697703</v>
+        <v>1841.8604651162791</v>
       </c>
       <c r="H100" s="3">
         <f t="shared" si="14"/>
-        <v>535.81395348837236</v>
+        <v>2210.2325581395353</v>
       </c>
       <c r="J100">
         <f t="shared" si="22"/>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="R100" s="3">
         <f t="shared" si="20"/>
-        <v>368.37209302325584</v>
+        <v>321.60000000000002</v>
       </c>
     </row>
     <row r="101" spans="5:18" x14ac:dyDescent="0.25">
@@ -5507,15 +5507,15 @@
       </c>
       <c r="F101" s="3">
         <f t="shared" si="12"/>
-        <v>360.93023255813972</v>
+        <v>1488.8372093023256</v>
       </c>
       <c r="G101" s="3">
         <f t="shared" si="13"/>
-        <v>451.16279069767472</v>
+        <v>1861.046511627907</v>
       </c>
       <c r="H101" s="3">
         <f t="shared" si="14"/>
-        <v>541.39534883720955</v>
+        <v>2233.2558139534885</v>
       </c>
       <c r="J101">
         <f t="shared" si="22"/>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="R101" s="3">
         <f t="shared" si="20"/>
-        <v>372.2093023255814</v>
+        <v>324.95</v>
       </c>
     </row>
     <row r="102" spans="5:18" x14ac:dyDescent="0.25">
@@ -5557,15 +5557,15 @@
       </c>
       <c r="F102" s="3">
         <f t="shared" si="12"/>
-        <v>364.65116279069787</v>
+        <v>1504.1860465116279</v>
       </c>
       <c r="G102" s="3">
         <f t="shared" si="13"/>
-        <v>455.81395348837236</v>
+        <v>1880.2325581395348</v>
       </c>
       <c r="H102" s="3">
         <f t="shared" si="14"/>
-        <v>546.97674418604674</v>
+        <v>2256.2790697674423</v>
       </c>
       <c r="J102">
         <f t="shared" si="22"/>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="R102" s="3">
         <f t="shared" si="20"/>
-        <v>376.04651162790697</v>
+        <v>328.3</v>
       </c>
     </row>
     <row r="103" spans="5:18" x14ac:dyDescent="0.25">
@@ -5607,15 +5607,15 @@
       </c>
       <c r="F103" s="3">
         <f t="shared" si="12"/>
-        <v>368.37209302325601</v>
+        <v>1519.5348837209303</v>
       </c>
       <c r="G103" s="3">
         <f t="shared" si="13"/>
-        <v>460.46511627907006</v>
+        <v>1899.4186046511629</v>
       </c>
       <c r="H103" s="3">
         <f t="shared" si="14"/>
-        <v>552.55813953488405</v>
+        <v>2279.3023255813955</v>
       </c>
       <c r="J103">
         <f t="shared" si="22"/>
@@ -5647,7 +5647,7 @@
       </c>
       <c r="R103" s="3">
         <f t="shared" si="20"/>
-        <v>379.88372093023258</v>
+        <v>331.65000000000003</v>
       </c>
     </row>
     <row r="104" spans="5:18" x14ac:dyDescent="0.25">
@@ -5657,15 +5657,15 @@
       </c>
       <c r="F104" s="3">
         <f t="shared" si="12"/>
-        <v>372.09302325581416</v>
+        <v>1534.8837209302326</v>
       </c>
       <c r="G104" s="3">
         <f t="shared" si="13"/>
-        <v>465.11627906976776</v>
+        <v>1918.6046511627908</v>
       </c>
       <c r="H104" s="3">
         <f t="shared" si="14"/>
-        <v>558.13953488372124</v>
+        <v>2302.3255813953492</v>
       </c>
       <c r="J104">
         <f t="shared" si="22"/>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="R104" s="3">
         <f t="shared" si="20"/>
-        <v>383.72093023255815</v>
+        <v>335</v>
       </c>
     </row>
     <row r="105" spans="5:18" x14ac:dyDescent="0.25">
@@ -5707,15 +5707,15 @@
       </c>
       <c r="F105" s="3">
         <f t="shared" si="12"/>
-        <v>375.81395348837231</v>
+        <v>1550.2325581395351</v>
       </c>
       <c r="G105" s="3">
         <f t="shared" si="13"/>
-        <v>469.7674418604654</v>
+        <v>1937.7906976744187</v>
       </c>
       <c r="H105" s="3">
         <f t="shared" si="14"/>
-        <v>563.72093023255843</v>
+        <v>2325.3488372093025</v>
       </c>
       <c r="J105">
         <f t="shared" si="22"/>
@@ -5747,7 +5747,7 @@
       </c>
       <c r="R105" s="3">
         <f t="shared" si="20"/>
-        <v>387.55813953488376</v>
+        <v>338.35</v>
       </c>
     </row>
     <row r="106" spans="5:18" x14ac:dyDescent="0.25">
@@ -5757,15 +5757,15 @@
       </c>
       <c r="F106" s="3">
         <f t="shared" si="12"/>
-        <v>379.53488372093045</v>
+        <v>1565.5813953488373</v>
       </c>
       <c r="G106" s="3">
         <f t="shared" si="13"/>
-        <v>474.41860465116309</v>
+        <v>1956.9767441860465</v>
       </c>
       <c r="H106" s="3">
         <f t="shared" si="14"/>
-        <v>569.30232558139562</v>
+        <v>2348.3720930232562</v>
       </c>
       <c r="J106">
         <f t="shared" si="22"/>
@@ -5797,7 +5797,7 @@
       </c>
       <c r="R106" s="3">
         <f t="shared" si="20"/>
-        <v>391.39534883720933</v>
+        <v>341.7</v>
       </c>
     </row>
     <row r="107" spans="5:18" x14ac:dyDescent="0.25">
@@ -5807,15 +5807,15 @@
       </c>
       <c r="F107" s="3">
         <f t="shared" si="12"/>
-        <v>383.2558139534886</v>
+        <v>1580.9302325581396</v>
       </c>
       <c r="G107" s="3">
         <f t="shared" si="13"/>
-        <v>479.06976744186079</v>
+        <v>1976.1627906976744</v>
       </c>
       <c r="H107" s="3">
         <f t="shared" si="14"/>
-        <v>574.88372093023281</v>
+        <v>2371.3953488372094</v>
       </c>
       <c r="J107">
         <f t="shared" si="22"/>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="R107" s="3">
         <f t="shared" si="20"/>
-        <v>395.23255813953489</v>
+        <v>345.05</v>
       </c>
     </row>
     <row r="108" spans="5:18" x14ac:dyDescent="0.25">
@@ -5857,15 +5857,15 @@
       </c>
       <c r="F108" s="3">
         <f t="shared" si="12"/>
-        <v>386.97674418604674</v>
+        <v>1596.279069767442</v>
       </c>
       <c r="G108" s="3">
         <f t="shared" si="13"/>
-        <v>483.72093023255843</v>
+        <v>1995.3488372093025</v>
       </c>
       <c r="H108" s="3">
         <f t="shared" si="14"/>
-        <v>580.46511627907012</v>
+        <v>2394.4186046511632</v>
       </c>
       <c r="J108">
         <f t="shared" si="22"/>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="R108" s="3">
         <f t="shared" si="20"/>
-        <v>399.06976744186051</v>
+        <v>348.40000000000003</v>
       </c>
     </row>
     <row r="109" spans="5:18" x14ac:dyDescent="0.25">
@@ -5907,15 +5907,15 @@
       </c>
       <c r="F109" s="3">
         <f t="shared" si="12"/>
-        <v>390.69767441860489</v>
+        <v>1611.6279069767443</v>
       </c>
       <c r="G109" s="3">
         <f t="shared" si="13"/>
-        <v>488.37209302325613</v>
+        <v>2014.5348837209303</v>
       </c>
       <c r="H109" s="3">
         <f t="shared" si="14"/>
-        <v>586.04651162790731</v>
+        <v>2417.4418604651164</v>
       </c>
       <c r="J109">
         <f t="shared" si="22"/>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="R109" s="3">
         <f t="shared" si="20"/>
-        <v>402.90697674418607</v>
+        <v>351.75</v>
       </c>
     </row>
     <row r="110" spans="5:18" x14ac:dyDescent="0.25">
@@ -5957,15 +5957,15 @@
       </c>
       <c r="F110" s="3">
         <f t="shared" si="12"/>
-        <v>394.41860465116304</v>
+        <v>1626.9767441860465</v>
       </c>
       <c r="G110" s="3">
         <f t="shared" si="13"/>
-        <v>493.02325581395382</v>
+        <v>2033.7209302325582</v>
       </c>
       <c r="H110" s="3">
         <f t="shared" si="14"/>
-        <v>591.6279069767445</v>
+        <v>2440.4651162790701</v>
       </c>
       <c r="J110">
         <f t="shared" si="22"/>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="R110" s="3">
         <f t="shared" si="20"/>
-        <v>406.74418604651163</v>
+        <v>355.1</v>
       </c>
     </row>
     <row r="111" spans="5:18" x14ac:dyDescent="0.25">
@@ -6007,15 +6007,15 @@
       </c>
       <c r="F111" s="3">
         <f t="shared" si="12"/>
-        <v>398.13953488372118</v>
+        <v>1642.325581395349</v>
       </c>
       <c r="G111" s="3">
         <f t="shared" si="13"/>
-        <v>497.67441860465146</v>
+        <v>2052.9069767441861</v>
       </c>
       <c r="H111" s="3">
         <f t="shared" si="14"/>
-        <v>597.20930232558169</v>
+        <v>2463.4883720930234</v>
       </c>
       <c r="J111">
         <f t="shared" si="22"/>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="R111" s="3">
         <f t="shared" si="20"/>
-        <v>410.58139534883725</v>
+        <v>358.45</v>
       </c>
     </row>
     <row r="112" spans="5:18" x14ac:dyDescent="0.25">
@@ -6057,15 +6057,15 @@
       </c>
       <c r="F112" s="3">
         <f t="shared" si="12"/>
-        <v>401.86046511627933</v>
+        <v>1657.6744186046512</v>
       </c>
       <c r="G112" s="3">
         <f t="shared" si="13"/>
-        <v>502.32558139534916</v>
+        <v>2072.0930232558139</v>
       </c>
       <c r="H112" s="3">
         <f t="shared" si="14"/>
-        <v>602.79069767441888</v>
+        <v>2486.5116279069771</v>
       </c>
       <c r="J112">
         <f t="shared" si="22"/>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="R112" s="3">
         <f t="shared" si="20"/>
-        <v>414.41860465116281</v>
+        <v>361.8</v>
       </c>
     </row>
     <row r="113" spans="5:18" x14ac:dyDescent="0.25">
@@ -6107,15 +6107,15 @@
       </c>
       <c r="F113" s="3">
         <f t="shared" si="12"/>
-        <v>405.58139534883742</v>
+        <v>1673.0232558139535</v>
       </c>
       <c r="G113" s="3">
         <f t="shared" si="13"/>
-        <v>506.97674418604686</v>
+        <v>2091.2790697674418</v>
       </c>
       <c r="H113" s="3">
         <f t="shared" si="14"/>
-        <v>608.37209302325607</v>
+        <v>2509.5348837209303</v>
       </c>
       <c r="J113">
         <f t="shared" si="22"/>
@@ -6147,7 +6147,7 @@
       </c>
       <c r="R113" s="3">
         <f t="shared" si="20"/>
-        <v>418.25581395348837</v>
+        <v>365.15000000000003</v>
       </c>
     </row>
     <row r="114" spans="5:18" x14ac:dyDescent="0.25">
@@ -6157,15 +6157,15 @@
       </c>
       <c r="F114" s="3">
         <f t="shared" si="12"/>
-        <v>409.30232558139556</v>
+        <v>1688.372093023256</v>
       </c>
       <c r="G114" s="3">
         <f t="shared" si="13"/>
-        <v>511.6279069767445</v>
+        <v>2110.4651162790697</v>
       </c>
       <c r="H114" s="3">
         <f t="shared" si="14"/>
-        <v>613.95348837209337</v>
+        <v>2532.558139534884</v>
       </c>
       <c r="J114">
         <f t="shared" si="22"/>
@@ -6197,7 +6197,7 @@
       </c>
       <c r="R114" s="3">
         <f t="shared" si="20"/>
-        <v>422.09302325581399</v>
+        <v>368.5</v>
       </c>
     </row>
     <row r="115" spans="5:18" x14ac:dyDescent="0.25">
@@ -6207,15 +6207,15 @@
       </c>
       <c r="F115" s="3">
         <f t="shared" si="12"/>
-        <v>413.02325581395371</v>
+        <v>1703.7209302325582</v>
       </c>
       <c r="G115" s="3">
         <f t="shared" si="13"/>
-        <v>516.27906976744214</v>
+        <v>2129.6511627906975</v>
       </c>
       <c r="H115" s="3">
         <f t="shared" si="14"/>
-        <v>619.53488372093057</v>
+        <v>2555.5813953488373</v>
       </c>
       <c r="J115">
         <f t="shared" si="22"/>
@@ -6247,7 +6247,7 @@
       </c>
       <c r="R115" s="3">
         <f t="shared" si="20"/>
-        <v>425.93023255813955</v>
+        <v>371.85</v>
       </c>
     </row>
     <row r="116" spans="5:18" x14ac:dyDescent="0.25">
@@ -6257,15 +6257,15 @@
       </c>
       <c r="F116" s="3">
         <f t="shared" si="12"/>
-        <v>416.74418604651186</v>
+        <v>1719.0697674418604</v>
       </c>
       <c r="G116" s="3">
         <f t="shared" si="13"/>
-        <v>520.93023255813989</v>
+        <v>2148.8372093023254</v>
       </c>
       <c r="H116" s="3">
         <f t="shared" si="14"/>
-        <v>625.11627906976776</v>
+        <v>2578.604651162791</v>
       </c>
       <c r="J116">
         <f t="shared" si="22"/>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="R116" s="3">
         <f t="shared" si="20"/>
-        <v>429.76744186046511</v>
+        <v>375.2</v>
       </c>
     </row>
     <row r="117" spans="5:18" x14ac:dyDescent="0.25">
@@ -6307,15 +6307,15 @@
       </c>
       <c r="F117" s="3">
         <f t="shared" si="12"/>
-        <v>420.46511627907</v>
+        <v>1734.4186046511629</v>
       </c>
       <c r="G117" s="3">
         <f t="shared" si="13"/>
-        <v>525.58139534883753</v>
+        <v>2168.0232558139537</v>
       </c>
       <c r="H117" s="3">
         <f t="shared" si="14"/>
-        <v>630.69767441860495</v>
+        <v>2601.6279069767443</v>
       </c>
       <c r="J117">
         <f t="shared" si="22"/>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="R117" s="3">
         <f t="shared" si="20"/>
-        <v>433.60465116279073</v>
+        <v>378.55</v>
       </c>
     </row>
     <row r="118" spans="5:18" x14ac:dyDescent="0.25">
@@ -6357,15 +6357,15 @@
       </c>
       <c r="F118" s="3">
         <f t="shared" si="12"/>
-        <v>424.18604651162815</v>
+        <v>1749.7674418604652</v>
       </c>
       <c r="G118" s="3">
         <f t="shared" si="13"/>
-        <v>530.23255813953517</v>
+        <v>2187.2093023255816</v>
       </c>
       <c r="H118" s="3">
         <f t="shared" si="14"/>
-        <v>636.27906976744214</v>
+        <v>2624.651162790698</v>
       </c>
       <c r="J118">
         <f t="shared" si="22"/>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="R118" s="3">
         <f t="shared" si="20"/>
-        <v>437.44186046511629</v>
+        <v>381.90000000000003</v>
       </c>
     </row>
     <row r="119" spans="5:18" x14ac:dyDescent="0.25">
@@ -6407,15 +6407,15 @@
       </c>
       <c r="F119" s="3">
         <f t="shared" si="12"/>
-        <v>427.9069767441863</v>
+        <v>1765.1162790697674</v>
       </c>
       <c r="G119" s="3">
         <f t="shared" si="13"/>
-        <v>534.88372093023293</v>
+        <v>2206.3953488372094</v>
       </c>
       <c r="H119" s="3">
         <f t="shared" si="14"/>
-        <v>641.86046511627944</v>
+        <v>2647.6744186046512</v>
       </c>
       <c r="J119">
         <f t="shared" si="22"/>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="R119" s="3">
         <f t="shared" si="20"/>
-        <v>441.27906976744185</v>
+        <v>385.25</v>
       </c>
     </row>
     <row r="120" spans="5:18" x14ac:dyDescent="0.25">
@@ -6457,15 +6457,15 @@
       </c>
       <c r="F120" s="3">
         <f t="shared" si="12"/>
-        <v>431.62790697674444</v>
+        <v>1780.4651162790699</v>
       </c>
       <c r="G120" s="3">
         <f t="shared" si="13"/>
-        <v>539.53488372093057</v>
+        <v>2225.5813953488373</v>
       </c>
       <c r="H120" s="3">
         <f t="shared" si="14"/>
-        <v>647.44186046511663</v>
+        <v>2670.6976744186049</v>
       </c>
       <c r="J120">
         <f t="shared" si="22"/>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="R120" s="3">
         <f t="shared" si="20"/>
-        <v>445.11627906976747</v>
+        <v>388.6</v>
       </c>
     </row>
     <row r="121" spans="5:18" x14ac:dyDescent="0.25">
@@ -6507,15 +6507,15 @@
       </c>
       <c r="F121" s="3">
         <f t="shared" si="12"/>
-        <v>435.34883720930259</v>
+        <v>1795.8139534883721</v>
       </c>
       <c r="G121" s="3">
         <f t="shared" si="13"/>
-        <v>544.18604651162821</v>
+        <v>2244.7674418604652</v>
       </c>
       <c r="H121" s="3">
         <f t="shared" si="14"/>
-        <v>653.02325581395382</v>
+        <v>2693.7209302325582</v>
       </c>
       <c r="J121">
         <f t="shared" si="22"/>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="R121" s="3">
         <f t="shared" si="20"/>
-        <v>448.95348837209303</v>
+        <v>391.95</v>
       </c>
     </row>
     <row r="122" spans="5:18" x14ac:dyDescent="0.25">
@@ -6557,15 +6557,15 @@
       </c>
       <c r="F122" s="3">
         <f t="shared" si="12"/>
-        <v>439.06976744186073</v>
+        <v>1811.1627906976744</v>
       </c>
       <c r="G122" s="3">
         <f t="shared" si="13"/>
-        <v>548.83720930232596</v>
+        <v>2263.953488372093</v>
       </c>
       <c r="H122" s="3">
         <f t="shared" si="14"/>
-        <v>658.60465116279101</v>
+        <v>2716.7441860465119</v>
       </c>
       <c r="J122">
         <f t="shared" si="22"/>
@@ -6597,7 +6597,7 @@
       </c>
       <c r="R122" s="3">
         <f t="shared" si="20"/>
-        <v>452.7906976744186</v>
+        <v>395.3</v>
       </c>
     </row>
     <row r="123" spans="5:18" x14ac:dyDescent="0.25">
@@ -6607,15 +6607,15 @@
       </c>
       <c r="F123" s="3">
         <f t="shared" si="12"/>
-        <v>442.79069767441888</v>
+        <v>1826.5116279069769</v>
       </c>
       <c r="G123" s="3">
         <f t="shared" si="13"/>
-        <v>553.4883720930236</v>
+        <v>2283.1395348837209</v>
       </c>
       <c r="H123" s="3">
         <f t="shared" si="14"/>
-        <v>664.18604651162821</v>
+        <v>2739.7674418604652</v>
       </c>
       <c r="J123">
         <f t="shared" si="22"/>
@@ -6647,7 +6647,7 @@
       </c>
       <c r="R123" s="3">
         <f t="shared" si="20"/>
-        <v>456.62790697674421</v>
+        <v>398.65000000000003</v>
       </c>
     </row>
     <row r="124" spans="5:18" x14ac:dyDescent="0.25">
@@ -6657,15 +6657,15 @@
       </c>
       <c r="F124" s="3">
         <f t="shared" si="12"/>
-        <v>446.51162790697703</v>
+        <v>1841.8604651162791</v>
       </c>
       <c r="G124" s="3">
         <f t="shared" si="13"/>
-        <v>558.13953488372124</v>
+        <v>2302.3255813953488</v>
       </c>
       <c r="H124" s="3">
         <f t="shared" si="14"/>
-        <v>669.7674418604654</v>
+        <v>2762.7906976744189</v>
       </c>
       <c r="J124">
         <f t="shared" si="22"/>
@@ -6697,7 +6697,7 @@
       </c>
       <c r="R124" s="3">
         <f t="shared" si="20"/>
-        <v>460.46511627906978</v>
+        <v>402</v>
       </c>
     </row>
     <row r="125" spans="5:18" x14ac:dyDescent="0.25">

</xml_diff>